<commit_message>
update GIE LNG list for collecting new terminals
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/01_raw/01_Russian_War_Case/2211_GIE_LNG_Database_public_updated.xlsx
+++ b/01_data/01_input_data/01_raw/01_Russian_War_Case/2211_GIE_LNG_Database_public_updated.xlsx
@@ -1,27 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{795C78A5-E2DC-458F-B4F6-1697F3A782FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258C9984-E97A-40D2-B571-4F1D4843FA20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5070" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import Terminals" sheetId="2" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="27" r:id="rId2"/>
-    <sheet name="Export Terminals" sheetId="26" r:id="rId3"/>
-    <sheet name="statistics" sheetId="25" r:id="rId4"/>
+    <sheet name="new_terminals" sheetId="28" r:id="rId3"/>
+    <sheet name="Export Terminals" sheetId="26" r:id="rId4"/>
+    <sheet name="statistics" sheetId="25" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Export Terminals'!$A$3:$H$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Export Terminals'!$A$3:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Import Terminals'!$A$3:$T$72</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">statistics!#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">statistics!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -357,7 +358,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="793" uniqueCount="274">
   <si>
     <t>Country</t>
   </si>
@@ -1329,6 +1330,21 @@
   </si>
   <si>
     <t>including planned</t>
+  </si>
+  <si>
+    <t>location</t>
+  </si>
+  <si>
+    <t>capacity</t>
+  </si>
+  <si>
+    <t>year in operation or build</t>
+  </si>
+  <si>
+    <t>source</t>
+  </si>
+  <si>
+    <t>part of previous list [yes/no]</t>
   </si>
 </sst>
 </file>
@@ -2523,6 +2539,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="5" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2532,7 +2549,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="17">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -2776,6 +2792,21 @@
     <tableColumn id="4" xr3:uid="{DDBD07BE-485B-40C9-8B3C-297E40133B83}" name="including planned" dataDxfId="0">
       <calculatedColumnFormula>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</calculatedColumnFormula>
     </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{EBDAC37A-2718-44DB-95E2-057AB1227D2B}" name="Table2" displayName="Table2" ref="A1:F3" totalsRowShown="0">
+  <autoFilter ref="A1:F3" xr:uid="{EBDAC37A-2718-44DB-95E2-057AB1227D2B}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{9A93E4EA-F484-4FCB-8E73-CF34F7541B67}" name="Country"/>
+    <tableColumn id="2" xr3:uid="{DD2FD98C-D8D7-4BDB-A198-D8301AD3704C}" name="location"/>
+    <tableColumn id="3" xr3:uid="{DBA0FB9F-2A2F-4690-B0FC-4F3287658968}" name="part of previous list [yes/no]"/>
+    <tableColumn id="4" xr3:uid="{F3FC3E39-C24E-4502-9637-E4521F948835}" name="capacity"/>
+    <tableColumn id="5" xr3:uid="{B56F1381-892D-4E87-9570-8E064DDAB8C5}" name="year in operation or build"/>
+    <tableColumn id="6" xr3:uid="{C95007E1-717A-4FF3-8F6C-3E1F2E38ACC4}" name="source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6718,15 +6749,15 @@
       <c r="B2" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="145">
+      <c r="C2" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>0</v>
       </c>
-      <c r="D2" s="145">
+      <c r="D2" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>0</v>
       </c>
-      <c r="E2" s="145">
+      <c r="E2" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>0</v>
       </c>
@@ -6735,15 +6766,15 @@
       <c r="B3" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="145">
+      <c r="C3" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>11.4</v>
       </c>
-      <c r="D3" s="145">
+      <c r="D3" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>15.3</v>
       </c>
-      <c r="E3" s="145">
+      <c r="E3" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>15.3</v>
       </c>
@@ -6752,15 +6783,15 @@
       <c r="B4" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="145">
+      <c r="C4" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>2.6</v>
       </c>
-      <c r="D4" s="145">
+      <c r="D4" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>2.6</v>
       </c>
-      <c r="E4" s="145">
+      <c r="E4" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>5.2</v>
       </c>
@@ -6769,15 +6800,15 @@
       <c r="B5" t="s">
         <v>43</v>
       </c>
-      <c r="C5" s="145">
+      <c r="C5" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>0</v>
       </c>
-      <c r="D5" s="145">
+      <c r="D5" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>2.44</v>
       </c>
-      <c r="E5" s="145">
+      <c r="E5" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>2.44</v>
       </c>
@@ -6786,15 +6817,15 @@
       <c r="B6" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="145">
+      <c r="C6" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>7.8</v>
       </c>
-      <c r="D6" s="145">
+      <c r="D6" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>7.8</v>
       </c>
-      <c r="E6" s="145">
+      <c r="E6" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>7.8</v>
       </c>
@@ -6803,15 +6834,15 @@
       <c r="B7" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="145">
+      <c r="C7" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>0</v>
       </c>
-      <c r="D7" s="145">
+      <c r="D7" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>0</v>
       </c>
-      <c r="E7" s="145">
+      <c r="E7" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>2.5</v>
       </c>
@@ -6820,15 +6851,15 @@
       <c r="B8" t="s">
         <v>60</v>
       </c>
-      <c r="C8" s="145">
+      <c r="C8" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>0</v>
       </c>
-      <c r="D8" s="145">
+      <c r="D8" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>0</v>
       </c>
-      <c r="E8" s="145">
+      <c r="E8" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>5</v>
       </c>
@@ -6837,15 +6868,15 @@
       <c r="B9" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="145">
+      <c r="C9" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>33</v>
       </c>
-      <c r="D9" s="145">
+      <c r="D9" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>33</v>
       </c>
-      <c r="E9" s="145">
+      <c r="E9" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>36.5</v>
       </c>
@@ -6854,15 +6885,15 @@
       <c r="B10" t="s">
         <v>77</v>
       </c>
-      <c r="C10" s="145">
+      <c r="C10" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>0</v>
       </c>
-      <c r="D10" s="145">
+      <c r="D10" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>0</v>
       </c>
-      <c r="E10" s="145">
+      <c r="E10" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>31.2</v>
       </c>
@@ -6871,15 +6902,15 @@
       <c r="B11" t="s">
         <v>92</v>
       </c>
-      <c r="C11" s="145">
+      <c r="C11" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>7</v>
       </c>
-      <c r="D11" s="145">
+      <c r="D11" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>12.5</v>
       </c>
-      <c r="E11" s="145">
+      <c r="E11" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>20.2</v>
       </c>
@@ -6888,15 +6919,15 @@
       <c r="B12" t="s">
         <v>105</v>
       </c>
-      <c r="C12" s="145">
+      <c r="C12" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>0</v>
       </c>
-      <c r="D12" s="145">
+      <c r="D12" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>0</v>
       </c>
-      <c r="E12" s="145">
+      <c r="E12" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>2.6</v>
       </c>
@@ -6905,15 +6936,15 @@
       <c r="B13" t="s">
         <v>112</v>
       </c>
-      <c r="C13" s="145">
+      <c r="C13" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>2.5</v>
       </c>
-      <c r="D13" s="145">
+      <c r="D13" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>2.5</v>
       </c>
-      <c r="E13" s="145">
+      <c r="E13" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>2.5</v>
       </c>
@@ -6922,15 +6953,15 @@
       <c r="B14" t="s">
         <v>116</v>
       </c>
-      <c r="C14" s="145">
+      <c r="C14" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>15.95</v>
       </c>
-      <c r="D14" s="145">
+      <c r="D14" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>15.95</v>
       </c>
-      <c r="E14" s="145">
+      <c r="E14" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>25.95</v>
       </c>
@@ -6939,15 +6970,15 @@
       <c r="B15" t="s">
         <v>133</v>
       </c>
-      <c r="C15" s="145">
+      <c r="C15" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>0</v>
       </c>
-      <c r="D15" s="145">
+      <c r="D15" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>0</v>
       </c>
-      <c r="E15" s="145">
+      <c r="E15" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>1.5</v>
       </c>
@@ -6956,15 +6987,15 @@
       <c r="B16" t="s">
         <v>138</v>
       </c>
-      <c r="C16" s="145">
+      <c r="C16" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>4</v>
       </c>
-      <c r="D16" s="145">
+      <c r="D16" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>4</v>
       </c>
-      <c r="E16" s="145">
+      <c r="E16" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>4</v>
       </c>
@@ -6973,15 +7004,15 @@
       <c r="B17" t="s">
         <v>142</v>
       </c>
-      <c r="C17" s="145">
+      <c r="C17" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>0.7</v>
       </c>
-      <c r="D17" s="145">
+      <c r="D17" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>0.7</v>
       </c>
-      <c r="E17" s="145">
+      <c r="E17" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>0.7</v>
       </c>
@@ -6990,15 +7021,15 @@
       <c r="B18" t="s">
         <v>146</v>
       </c>
-      <c r="C18" s="145">
+      <c r="C18" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>0</v>
       </c>
-      <c r="D18" s="145">
+      <c r="D18" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>0</v>
       </c>
-      <c r="E18" s="145">
+      <c r="E18" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>3</v>
       </c>
@@ -7007,15 +7038,15 @@
       <c r="B19" t="s">
         <v>153</v>
       </c>
-      <c r="C19" s="145">
+      <c r="C19" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>12</v>
       </c>
-      <c r="D19" s="145">
+      <c r="D19" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>21.5</v>
       </c>
-      <c r="E19" s="145">
+      <c r="E19" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>24</v>
       </c>
@@ -7024,15 +7055,15 @@
       <c r="B20" t="s">
         <v>161</v>
       </c>
-      <c r="C20" s="145">
+      <c r="C20" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>6.2</v>
       </c>
-      <c r="D20" s="145">
+      <c r="D20" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>8.3000000000000007</v>
       </c>
-      <c r="E20" s="145">
+      <c r="E20" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>14.4</v>
       </c>
@@ -7041,15 +7072,15 @@
       <c r="B21" t="s">
         <v>166</v>
       </c>
-      <c r="C21" s="145">
+      <c r="C21" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>7.6</v>
       </c>
-      <c r="D21" s="145">
+      <c r="D21" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>7.6</v>
       </c>
-      <c r="E21" s="145">
+      <c r="E21" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>7.6</v>
       </c>
@@ -7058,15 +7089,15 @@
       <c r="B22" t="s">
         <v>170</v>
       </c>
-      <c r="C22" s="145">
+      <c r="C22" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>3.7</v>
       </c>
-      <c r="D22" s="145">
+      <c r="D22" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>3.7</v>
       </c>
-      <c r="E22" s="145">
+      <c r="E22" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>3.7</v>
       </c>
@@ -7075,15 +7106,15 @@
       <c r="B23" t="s">
         <v>174</v>
       </c>
-      <c r="C23" s="145">
+      <c r="C23" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>60.100000000000009</v>
       </c>
-      <c r="D23" s="145">
+      <c r="D23" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>60.100000000000009</v>
       </c>
-      <c r="E23" s="145">
+      <c r="E23" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>60.100000000000009</v>
       </c>
@@ -7092,15 +7123,15 @@
       <c r="B24" t="s">
         <v>191</v>
       </c>
-      <c r="C24" s="145">
+      <c r="C24" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>43.6</v>
       </c>
-      <c r="D24" s="145">
+      <c r="D24" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>43.6</v>
       </c>
-      <c r="E24" s="145">
+      <c r="E24" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>53.3</v>
       </c>
@@ -7109,15 +7140,15 @@
       <c r="B25" t="s">
         <v>203</v>
       </c>
-      <c r="C25" s="145">
+      <c r="C25" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</f>
         <v>48.1</v>
       </c>
-      <c r="D25" s="145">
+      <c r="D25" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
         <v>53.1</v>
       </c>
-      <c r="E25" s="145">
+      <c r="E25" s="142">
         <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>53.1</v>
       </c>
@@ -7131,6 +7162,46 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2E2D5C9-6454-49C3-A8E3-C7067161AA7F}">
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.7265625" customWidth="1"/>
+    <col min="2" max="2" width="9.6328125" customWidth="1"/>
+    <col min="3" max="3" width="27.1796875" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="24.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>269</v>
+      </c>
+      <c r="C1" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1" t="s">
+        <v>270</v>
+      </c>
+      <c r="E1" t="s">
+        <v>271</v>
+      </c>
+      <c r="F1" t="s">
+        <v>272</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0AA7DE4-CF5E-4E90-9185-90533C419FFC}">
   <sheetPr>
     <tabColor rgb="FF246A31"/>
@@ -7151,11 +7222,11 @@
   <sheetData>
     <row r="1" spans="1:21" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="117"/>
-      <c r="C1" s="142" t="s">
+      <c r="C1" s="143" t="s">
         <v>265</v>
       </c>
-      <c r="D1" s="143"/>
-      <c r="E1" s="143"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
     </row>
     <row r="2" spans="1:21" ht="13" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C2" s="118"/>
@@ -7507,7 +7578,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8BD7156-22F1-468E-9BDE-E7129A7A2251}">
   <sheetPr codeName="Sheet3">
     <pageSetUpPr fitToPage="1"/>
@@ -7526,24 +7597,24 @@
   <sheetData>
     <row r="1" spans="2:8" ht="61.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:8" ht="13" x14ac:dyDescent="0.25">
-      <c r="B2" s="144" t="s">
+      <c r="B2" s="145" t="s">
         <v>218</v>
       </c>
-      <c r="C2" s="144"/>
-      <c r="D2" s="144"/>
-      <c r="E2" s="144"/>
-      <c r="F2" s="144"/>
-      <c r="G2" s="144"/>
+      <c r="C2" s="145"/>
+      <c r="D2" s="145"/>
+      <c r="E2" s="145"/>
+      <c r="F2" s="145"/>
+      <c r="G2" s="145"/>
     </row>
     <row r="3" spans="2:8" ht="13" x14ac:dyDescent="0.25">
-      <c r="B3" s="144" t="s">
+      <c r="B3" s="145" t="s">
         <v>219</v>
       </c>
-      <c r="C3" s="144"/>
-      <c r="D3" s="144"/>
-      <c r="E3" s="144"/>
-      <c r="F3" s="144"/>
-      <c r="G3" s="144"/>
+      <c r="C3" s="145"/>
+      <c r="D3" s="145"/>
+      <c r="E3" s="145"/>
+      <c r="F3" s="145"/>
+      <c r="G3" s="145"/>
     </row>
     <row r="4" spans="2:8" ht="13" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="2:8" s="6" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -7947,14 +8018,14 @@
       <c r="G30" s="36"/>
     </row>
     <row r="32" spans="2:8" ht="13" x14ac:dyDescent="0.25">
-      <c r="B32" s="144" t="s">
+      <c r="B32" s="145" t="s">
         <v>229</v>
       </c>
-      <c r="C32" s="144"/>
-      <c r="D32" s="144"/>
-      <c r="E32" s="144"/>
-      <c r="F32" s="144"/>
-      <c r="G32" s="144"/>
+      <c r="C32" s="145"/>
+      <c r="D32" s="145"/>
+      <c r="E32" s="145"/>
+      <c r="F32" s="145"/>
+      <c r="G32" s="145"/>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="22"/>
@@ -8100,14 +8171,14 @@
       <c r="H42" s="37"/>
     </row>
     <row r="44" spans="2:8" ht="13" x14ac:dyDescent="0.25">
-      <c r="B44" s="144" t="s">
+      <c r="B44" s="145" t="s">
         <v>230</v>
       </c>
-      <c r="C44" s="144"/>
-      <c r="D44" s="144"/>
-      <c r="E44" s="144"/>
-      <c r="F44" s="144"/>
-      <c r="G44" s="144"/>
+      <c r="C44" s="145"/>
+      <c r="D44" s="145"/>
+      <c r="E44" s="145"/>
+      <c r="F44" s="145"/>
+      <c r="G44" s="145"/>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B45" s="22"/>
@@ -8265,14 +8336,14 @@
       <c r="H55" s="37"/>
     </row>
     <row r="58" spans="2:8" ht="13" x14ac:dyDescent="0.25">
-      <c r="B58" s="144" t="s">
+      <c r="B58" s="145" t="s">
         <v>231</v>
       </c>
-      <c r="C58" s="144"/>
-      <c r="D58" s="144"/>
-      <c r="E58" s="144"/>
-      <c r="F58" s="144"/>
-      <c r="G58" s="144"/>
+      <c r="C58" s="145"/>
+      <c r="D58" s="145"/>
+      <c r="E58" s="145"/>
+      <c r="F58" s="145"/>
+      <c r="G58" s="145"/>
     </row>
     <row r="59" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B59" s="22"/>
@@ -8430,14 +8501,14 @@
       <c r="G70" s="71"/>
     </row>
     <row r="72" spans="2:7" ht="13" x14ac:dyDescent="0.25">
-      <c r="B72" s="144" t="s">
+      <c r="B72" s="145" t="s">
         <v>232</v>
       </c>
-      <c r="C72" s="144"/>
-      <c r="D72" s="144"/>
-      <c r="E72" s="144"/>
-      <c r="F72" s="144"/>
-      <c r="G72" s="144"/>
+      <c r="C72" s="145"/>
+      <c r="D72" s="145"/>
+      <c r="E72" s="145"/>
+      <c r="F72" s="145"/>
+      <c r="G72" s="145"/>
     </row>
     <row r="73" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B73" s="22"/>
@@ -8623,6 +8694,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009E4146C62EF569408BE446968F8E2BB2" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="254593c6bb6e9a2bdf6bbb582ab27135">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="715071c2-35c6-41f1-a6a3-03dd21313204" xmlns:ns3="c2313526-4958-4054-bf54-a58bf530b099" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a1948b7e2db5dcbc8e8cadbefc825eb7" ns2:_="" ns3:_="">
     <xsd:import namespace="715071c2-35c6-41f1-a6a3-03dd21313204"/>
@@ -8817,15 +8897,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -8838,6 +8909,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD84AF24-CD79-4A30-B9DC-32ADB805B515}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E765955-317A-4E81-8365-42F9F8DFA40D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8852,14 +8931,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD84AF24-CD79-4A30-B9DC-32ADB805B515}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
add new GIE LNG data sheet and update inputs
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/01_raw/01_Russian_War_Case/2211_GIE_LNG_Database_public_updated.xlsx
+++ b/01_data/01_input_data/01_raw/01_Russian_War_Case/2211_GIE_LNG_Database_public_updated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258C9984-E97A-40D2-B571-4F1D4843FA20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51982F9-DFA9-4CF3-AB3E-F09D7A18811E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import Terminals" sheetId="2" r:id="rId1"/>
@@ -358,7 +358,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="793" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="794" uniqueCount="275">
   <si>
     <t>Country</t>
   </si>
@@ -1329,9 +1329,6 @@
     <t>including under construction</t>
   </si>
   <si>
-    <t>including planned</t>
-  </si>
-  <si>
     <t>location</t>
   </si>
   <si>
@@ -1345,6 +1342,12 @@
   </si>
   <si>
     <t>part of previous list [yes/no]</t>
+  </si>
+  <si>
+    <t>including planneduntil 2025</t>
+  </si>
+  <si>
+    <t>including planneduntil 2035</t>
   </si>
 </sst>
 </file>
@@ -2569,7 +2572,10 @@
     <cellStyle name="Normal 2 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
     <cellStyle name="Normal 3" xfId="7" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -2779,18 +2785,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DF730721-4E67-4389-BDEC-93D098A8839E}" name="Table1" displayName="Table1" ref="B1:E25" totalsRowShown="0">
-  <autoFilter ref="B1:E25" xr:uid="{DF730721-4E67-4389-BDEC-93D098A8839E}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DF730721-4E67-4389-BDEC-93D098A8839E}" name="Table1" displayName="Table1" ref="B1:F25" totalsRowShown="0">
+  <autoFilter ref="B1:F25" xr:uid="{DF730721-4E67-4389-BDEC-93D098A8839E}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{2B75C2E5-36CB-4CEB-A722-42C024E65199}" name="Country"/>
-    <tableColumn id="2" xr3:uid="{C0DC37A5-1451-4376-BDA9-CC92E20CB492}" name="Operational in 2021" dataDxfId="2">
+    <tableColumn id="2" xr3:uid="{C0DC37A5-1451-4376-BDA9-CC92E20CB492}" name="Operational in 2021" dataDxfId="3">
       <calculatedColumnFormula>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2022")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{45CE4E93-27C3-4D7C-B68C-AAE86B69F89D}" name="including under construction" dataDxfId="1">
-      <calculatedColumnFormula>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{45CE4E93-27C3-4D7C-B68C-AAE86B69F89D}" name="including under construction" dataDxfId="2">
+      <calculatedColumnFormula>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DDBD07BE-485B-40C9-8B3C-297E40133B83}" name="including planned" dataDxfId="0">
-      <calculatedColumnFormula>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</calculatedColumnFormula>
+    <tableColumn id="4" xr3:uid="{DDBD07BE-485B-40C9-8B3C-297E40133B83}" name="including planneduntil 2025" dataDxfId="1">
+      <calculatedColumnFormula>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{E3270E7B-5483-43EC-B275-40D5836373D4}" name="including planneduntil 2035" dataDxfId="0">
+      <calculatedColumnFormula>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3110,7 +3119,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr codeName="Sheet1">
+  <sheetPr codeName="Sheet1" filterMode="1">
     <tabColor rgb="FF0070C0"/>
   </sheetPr>
   <dimension ref="A1:U72"/>
@@ -3235,7 +3244,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="80" t="s">
         <v>20</v>
       </c>
@@ -3273,7 +3282,7 @@
       <c r="S4" s="81"/>
       <c r="T4" s="85"/>
     </row>
-    <row r="5" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="86" t="s">
         <v>27</v>
       </c>
@@ -3332,7 +3341,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="86" t="s">
         <v>27</v>
       </c>
@@ -3374,7 +3383,7 @@
       <c r="S6" s="92"/>
       <c r="T6" s="91"/>
     </row>
-    <row r="7" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="86" t="s">
         <v>27</v>
       </c>
@@ -3416,7 +3425,7 @@
       <c r="S7" s="92"/>
       <c r="T7" s="91"/>
     </row>
-    <row r="8" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="86" t="s">
         <v>38</v>
       </c>
@@ -3474,7 +3483,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:20" s="4" customFormat="1" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" s="4" customFormat="1" ht="13.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="93" t="s">
         <v>38</v>
       </c>
@@ -3532,7 +3541,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:20" s="4" customFormat="1" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" s="4" customFormat="1" ht="13.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="93" t="s">
         <v>43</v>
       </c>
@@ -3580,7 +3589,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="93" t="s">
         <v>48</v>
       </c>
@@ -3618,7 +3627,7 @@
       <c r="S11" s="95"/>
       <c r="T11" s="99"/>
     </row>
-    <row r="12" spans="1:20" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" s="4" customFormat="1" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="93" t="s">
         <v>48</v>
       </c>
@@ -3662,7 +3671,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="13" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="93" t="s">
         <v>55</v>
       </c>
@@ -3708,7 +3717,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:20" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" s="4" customFormat="1" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="86" t="s">
         <v>55</v>
       </c>
@@ -3750,7 +3759,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:20" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" s="4" customFormat="1" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="86" t="s">
         <v>60</v>
       </c>
@@ -3792,7 +3801,7 @@
       <c r="S15" s="102"/>
       <c r="T15" s="11"/>
     </row>
-    <row r="16" spans="1:20" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" s="4" customFormat="1" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="86" t="s">
         <v>63</v>
       </c>
@@ -3850,7 +3859,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="17" spans="1:21" s="4" customFormat="1" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" s="4" customFormat="1" ht="13.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="86" t="s">
         <v>63</v>
       </c>
@@ -3908,7 +3917,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="18" spans="1:21" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="86" t="s">
         <v>63</v>
       </c>
@@ -3954,7 +3963,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="19" spans="1:21" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" s="5" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="86" t="s">
         <v>63</v>
       </c>
@@ -4000,7 +4009,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:21" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="86" t="s">
         <v>63</v>
       </c>
@@ -4058,7 +4067,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="21" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="86" t="s">
         <v>63</v>
       </c>
@@ -4116,7 +4125,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="22" spans="1:21" s="35" customFormat="1" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" s="35" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="86" t="s">
         <v>63</v>
       </c>
@@ -4391,7 +4400,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="1:21" s="4" customFormat="1" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" s="4" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="86" t="s">
         <v>92</v>
       </c>
@@ -4435,7 +4444,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="29" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="93" t="s">
         <v>92</v>
       </c>
@@ -4489,7 +4498,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="30" spans="1:21" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" s="35" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="87" t="s">
         <v>92</v>
       </c>
@@ -4531,7 +4540,7 @@
       <c r="S30" s="87"/>
       <c r="T30" s="91"/>
     </row>
-    <row r="31" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="86" t="s">
         <v>92</v>
       </c>
@@ -4589,7 +4598,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="32" spans="1:21" s="35" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" s="35" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="86" t="s">
         <v>92</v>
       </c>
@@ -4635,7 +4644,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="33" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="93" t="s">
         <v>105</v>
       </c>
@@ -4675,7 +4684,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="34" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="93" t="s">
         <v>105</v>
       </c>
@@ -4717,7 +4726,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="35" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="86" t="s">
         <v>112</v>
       </c>
@@ -4761,7 +4770,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="36" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="86" t="s">
         <v>116</v>
       </c>
@@ -4819,7 +4828,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="37" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="86" t="s">
         <v>116</v>
       </c>
@@ -4877,7 +4886,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="38" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="86" t="s">
         <v>116</v>
       </c>
@@ -4923,7 +4932,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="39" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="86" t="s">
         <v>116</v>
       </c>
@@ -4969,7 +4978,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="40" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="93" t="s">
         <v>116</v>
       </c>
@@ -5020,7 +5029,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="41" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="86" t="s">
         <v>116</v>
       </c>
@@ -5078,7 +5087,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="42" spans="1:20" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="93" t="s">
         <v>133</v>
       </c>
@@ -5126,7 +5135,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="43" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="86" t="s">
         <v>138</v>
       </c>
@@ -5182,7 +5191,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="44" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="93" t="s">
         <v>142</v>
       </c>
@@ -5230,7 +5239,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="93" t="s">
         <v>146</v>
       </c>
@@ -5270,7 +5279,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="46" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="93" t="s">
         <v>146</v>
       </c>
@@ -5312,7 +5321,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="47" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="86" t="s">
         <v>153</v>
       </c>
@@ -5372,7 +5381,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="48" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="86" t="s">
         <v>153</v>
       </c>
@@ -5416,7 +5425,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="49" spans="1:21" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="86" t="s">
         <v>153</v>
       </c>
@@ -5466,7 +5475,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="50" spans="1:21" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="86" t="s">
         <v>153</v>
       </c>
@@ -5523,7 +5532,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="51" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="86" t="s">
         <v>161</v>
       </c>
@@ -5577,7 +5586,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="52" spans="1:21" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="86" t="s">
         <v>161</v>
       </c>
@@ -5635,7 +5644,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="53" spans="1:21" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="86" t="s">
         <v>161</v>
       </c>
@@ -5686,7 +5695,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="54" spans="1:21" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="86" t="s">
         <v>166</v>
       </c>
@@ -5744,7 +5753,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="55" spans="1:21" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="86" t="s">
         <v>170</v>
       </c>
@@ -5788,7 +5797,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="56" spans="1:21" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="86" t="s">
         <v>174</v>
       </c>
@@ -5846,7 +5855,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="57" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="86" t="s">
         <v>174</v>
       </c>
@@ -5904,7 +5913,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="58" spans="1:21" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="86" t="s">
         <v>174</v>
       </c>
@@ -5962,7 +5971,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="59" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="86" t="s">
         <v>174</v>
       </c>
@@ -6020,7 +6029,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="60" spans="1:21" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="86" t="s">
         <v>174</v>
       </c>
@@ -6078,7 +6087,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="61" spans="1:21" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="86" t="s">
         <v>174</v>
       </c>
@@ -6136,7 +6145,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="62" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="86" t="s">
         <v>174</v>
       </c>
@@ -6194,7 +6203,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="63" spans="1:21" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="86" t="s">
         <v>191</v>
       </c>
@@ -6244,7 +6253,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="64" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="86" t="s">
         <v>191</v>
       </c>
@@ -6294,7 +6303,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="65" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="86" t="s">
         <v>191</v>
       </c>
@@ -6338,7 +6347,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="66" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="86" t="s">
         <v>191</v>
       </c>
@@ -6382,7 +6391,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="67" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="86" t="s">
         <v>191</v>
       </c>
@@ -6432,7 +6441,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="68" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="86" t="s">
         <v>203</v>
       </c>
@@ -6490,7 +6499,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="69" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="86" t="s">
         <v>203</v>
       </c>
@@ -6539,7 +6548,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="70" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="86" t="s">
         <v>203</v>
       </c>
@@ -6597,7 +6606,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="71" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="86" t="s">
         <v>203</v>
       </c>
@@ -6655,7 +6664,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="72" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="86" t="s">
         <v>203</v>
       </c>
@@ -6705,6 +6714,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A3:T72" xr:uid="{E98519F1-1ABB-4F31-8F6B-DA296018CBA6}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Germany"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:T72">
       <sortCondition ref="A3:A72"/>
     </sortState>
@@ -6723,7 +6737,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F698641-434F-489E-899B-C15059196C75}">
-  <dimension ref="B1:E25"/>
+  <dimension ref="B1:F25"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12.54296875" customWidth="1"/>
@@ -6731,7 +6745,7 @@
     <col min="5" max="5" width="21.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -6742,10 +6756,13 @@
         <v>267</v>
       </c>
       <c r="E1" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+        <v>273</v>
+      </c>
+      <c r="F1" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>20</v>
       </c>
@@ -6754,15 +6771,19 @@
         <v>0</v>
       </c>
       <c r="D2" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>0</v>
       </c>
       <c r="E2" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F2" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>27</v>
       </c>
@@ -6771,15 +6792,19 @@
         <v>11.4</v>
       </c>
       <c r="D3" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>15.3</v>
       </c>
       <c r="E3" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>15.3</v>
       </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F3" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>15.3</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>38</v>
       </c>
@@ -6788,15 +6813,19 @@
         <v>2.6</v>
       </c>
       <c r="D4" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>2.6</v>
       </c>
       <c r="E4" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
+        <v>2.6</v>
+      </c>
+      <c r="F4" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>5.2</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>43</v>
       </c>
@@ -6805,15 +6834,19 @@
         <v>0</v>
       </c>
       <c r="D5" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>2.44</v>
       </c>
       <c r="E5" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>2.44</v>
       </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F5" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>2.44</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>48</v>
       </c>
@@ -6822,15 +6855,19 @@
         <v>7.8</v>
       </c>
       <c r="D6" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>7.8</v>
       </c>
       <c r="E6" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>7.8</v>
       </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F6" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>55</v>
       </c>
@@ -6839,15 +6876,19 @@
         <v>0</v>
       </c>
       <c r="D7" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>0</v>
       </c>
       <c r="E7" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>2.5</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>60</v>
       </c>
@@ -6856,15 +6897,19 @@
         <v>0</v>
       </c>
       <c r="D8" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>0</v>
       </c>
       <c r="E8" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F8" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>63</v>
       </c>
@@ -6873,15 +6918,19 @@
         <v>33</v>
       </c>
       <c r="D9" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>33</v>
       </c>
       <c r="E9" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
+        <v>34.5</v>
+      </c>
+      <c r="F9" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>36.5</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>77</v>
       </c>
@@ -6890,15 +6939,19 @@
         <v>0</v>
       </c>
       <c r="D10" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>0</v>
       </c>
       <c r="E10" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
+        <v>17</v>
+      </c>
+      <c r="F10" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>31.2</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>92</v>
       </c>
@@ -6907,15 +6960,19 @@
         <v>7</v>
       </c>
       <c r="D11" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>12.5</v>
       </c>
       <c r="E11" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>20.2</v>
       </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F11" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>20.2</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>105</v>
       </c>
@@ -6924,15 +6981,19 @@
         <v>0</v>
       </c>
       <c r="D12" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>0</v>
       </c>
       <c r="E12" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>2.6</v>
       </c>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F12" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>112</v>
       </c>
@@ -6941,15 +7002,19 @@
         <v>2.5</v>
       </c>
       <c r="D13" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>2.5</v>
       </c>
       <c r="E13" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>2.5</v>
       </c>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F13" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>116</v>
       </c>
@@ -6958,15 +7023,19 @@
         <v>15.95</v>
       </c>
       <c r="D14" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>15.95</v>
       </c>
       <c r="E14" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>25.95</v>
       </c>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F14" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>25.95</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>133</v>
       </c>
@@ -6975,15 +7044,19 @@
         <v>0</v>
       </c>
       <c r="D15" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>0</v>
       </c>
       <c r="E15" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>1.5</v>
       </c>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F15" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>138</v>
       </c>
@@ -6992,15 +7065,19 @@
         <v>4</v>
       </c>
       <c r="D16" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>4</v>
       </c>
       <c r="E16" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>4</v>
       </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F16" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>142</v>
       </c>
@@ -7009,15 +7086,19 @@
         <v>0.7</v>
       </c>
       <c r="D17" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>0.7</v>
       </c>
       <c r="E17" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>0.7</v>
       </c>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F17" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>146</v>
       </c>
@@ -7026,15 +7107,19 @@
         <v>0</v>
       </c>
       <c r="D18" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>0</v>
       </c>
       <c r="E18" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
+        <v>0</v>
+      </c>
+      <c r="F18" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>153</v>
       </c>
@@ -7043,15 +7128,19 @@
         <v>12</v>
       </c>
       <c r="D19" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>21.5</v>
       </c>
       <c r="E19" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
+        <v>21.5</v>
+      </c>
+      <c r="F19" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>161</v>
       </c>
@@ -7060,15 +7149,19 @@
         <v>6.2</v>
       </c>
       <c r="D20" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>8.3000000000000007</v>
       </c>
       <c r="E20" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="F20" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
         <v>14.4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>166</v>
       </c>
@@ -7077,15 +7170,19 @@
         <v>7.6</v>
       </c>
       <c r="D21" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>7.6</v>
       </c>
       <c r="E21" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>7.6</v>
       </c>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F21" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>170</v>
       </c>
@@ -7094,15 +7191,19 @@
         <v>3.7</v>
       </c>
       <c r="D22" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>3.7</v>
       </c>
       <c r="E22" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>3.7</v>
       </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F22" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>174</v>
       </c>
@@ -7111,15 +7212,19 @@
         <v>60.100000000000009</v>
       </c>
       <c r="D23" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>60.100000000000009</v>
       </c>
       <c r="E23" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>60.100000000000009</v>
       </c>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F23" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>60.100000000000009</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>191</v>
       </c>
@@ -7128,15 +7233,19 @@
         <v>43.6</v>
       </c>
       <c r="D24" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>43.6</v>
       </c>
       <c r="E24" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
         <v>53.3</v>
       </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F24" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>53.3</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>203</v>
       </c>
@@ -7145,12 +7254,16 @@
         <v>48.1</v>
       </c>
       <c r="D25" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")</f>
-        <v>53.1</v>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
+        <v>48.1</v>
       </c>
       <c r="E25" s="142">
-        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2026")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
-        <v>53.1</v>
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2025")</f>
+        <v>48.1</v>
+      </c>
+      <c r="F25" s="142">
+        <f>SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"operational",'Import Terminals'!$F$4:$F$72,"&lt;2024")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"under construction",'Import Terminals'!$F$4:$F$72,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$72,'Import Terminals'!$A$4:$A$72,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$72,"planned",'Import Terminals'!$F$4:$F$72,"&lt;2035")</f>
+        <v>48.1</v>
       </c>
     </row>
   </sheetData>
@@ -7178,19 +7291,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>268</v>
+      </c>
+      <c r="C1" t="s">
+        <v>272</v>
+      </c>
+      <c r="D1" t="s">
         <v>269</v>
       </c>
-      <c r="C1" t="s">
-        <v>273</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>270</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>271</v>
-      </c>
-      <c r="F1" t="s">
-        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -8694,15 +8807,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009E4146C62EF569408BE446968F8E2BB2" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="254593c6bb6e9a2bdf6bbb582ab27135">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="715071c2-35c6-41f1-a6a3-03dd21313204" xmlns:ns3="c2313526-4958-4054-bf54-a58bf530b099" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a1948b7e2db5dcbc8e8cadbefc825eb7" ns2:_="" ns3:_="">
     <xsd:import namespace="715071c2-35c6-41f1-a6a3-03dd21313204"/>
@@ -8897,6 +9001,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -8909,14 +9022,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD84AF24-CD79-4A30-B9DC-32ADB805B515}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E765955-317A-4E81-8365-42F9F8DFA40D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8931,6 +9036,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD84AF24-CD79-4A30-B9DC-32ADB805B515}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>